<commit_message>
up besar & fix bug
</commit_message>
<xml_diff>
--- a/laporan.xlsx
+++ b/laporan.xlsx
@@ -7,22 +7,90 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
-    <sheet name="Laporan" sheetId="1" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="2" r:id="rId4"/>
+    <sheet name="Barang" sheetId="3" r:id="rId6"/>
+    <sheet name="Transaksi" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+  <si>
+    <t>DASHBOARD TOKO</t>
+  </si>
+  <si>
+    <t>Saldo Toko</t>
+  </si>
+  <si>
+    <t>Total Penjualan</t>
+  </si>
+  <si>
+    <t>Total Penarikan</t>
+  </si>
+  <si>
+    <t>Total Transaksi</t>
+  </si>
+  <si>
+    <t>Barang Terjual</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
   <si>
     <t>Nama Barang</t>
   </si>
   <si>
-    <t>Jumlah Terjual</t>
+    <t>Kategori</t>
+  </si>
+  <si>
+    <t>Harga</t>
+  </si>
+  <si>
+    <t>Stok</t>
+  </si>
+  <si>
+    <t>Terjual</t>
   </si>
   <si>
     <t>btc</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>pensil</t>
+  </si>
+  <si>
+    <t>atk</t>
+  </si>
+  <si>
+    <t>pulpen</t>
+  </si>
+  <si>
+    <t>tas</t>
+  </si>
+  <si>
+    <t>perskl</t>
+  </si>
+  <si>
+    <t>Pembeli</t>
+  </si>
+  <si>
+    <t>Barang</t>
+  </si>
+  <si>
+    <t>Jumlah</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Pembayaran</t>
+  </si>
+  <si>
+    <t>Status</t>
   </si>
 </sst>
 </file>
@@ -88,7 +156,7 @@
                   <a:srgbClr val="595959"/>
                 </a:solidFill>
               </a:rPr>
-              <a:t>Grafik Penjualan Barang</a:t>
+              <a:t>Grafik Barang Terjual</a:t>
             </a:r>
             <a:endParaRPr lang="en-US" altLang="en-US"/>
           </a:p>
@@ -126,7 +194,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>Penjualan</f>
+              <f>Barang!$F$1</f>
             </strRef>
           </tx>
           <dLbls>
@@ -149,12 +217,12 @@
           <invertIfNegative val="0"/>
           <cat>
             <strRef>
-              <f>Laporan!$A$2:$A$20</f>
+              <f>Barang!$B$2:$B$5</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>Laporan!$B$2:$B$20</f>
+              <f>Barang!$F$2:$F$5</f>
               <numCache>
                 <formatCode/>
               </numCache>
@@ -289,16 +357,16 @@
 <xdr:wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -576,28 +644,195 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>2012000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
       <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
         <v>1</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>1000000000</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B2">
-        <v>37</v>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3">
+        <v>2000</v>
+      </c>
+      <c r="E3">
+        <v>22</v>
+      </c>
+      <c r="F3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4">
+        <v>5000</v>
+      </c>
+      <c r="E4">
+        <v>35</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5">
+        <v>1000000</v>
+      </c>
+      <c r="E5">
+        <v>10</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>